<commit_message>
Cloud Slippers AH26 : bascule sur une selection pilotee par les motifs
Agregation des 3 gros produits sur 12 mois : les motifs imprimes font 31% du
volume du chausson contre 9,4% de la chaussure, soit 3,3x. Les unis de saison
(Terracotta 6%, Burgundy 4,4%, Forest Green 3%) ne justifient pas une place.

Sortis : Terracotta, Burgundy Wine, Forest Green, Nordic Fair Isle, Espresso.
Entres : Black Leopard, Grey Leopard, Cow Print, Houndstooth.
Conserves : Heather Grey Marl, Grey Camo, Navy, Buffalo Check.

Black Leopard et Grey Leopard reutilisent l'artwork exact du Leopard Brown
deja en production : recoloration seule, aucun developpement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012DysLVZGD3n9nCQtdYE4Vz
</commit_message>
<xml_diff>
--- a/aw26-cloud-slippers/PO-CloudSlippers-AW26.xlsx
+++ b/aw26-cloud-slippers/PO-CloudSlippers-AW26.xlsx
@@ -85,7 +85,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -114,27 +114,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="009A9A9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00111111"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B9B7B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="008E9094"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009A9A9A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004A342A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B0603C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006E2233"/>
+        <fgColor rgb="00F2EFE9"/>
       </patternFill>
     </fill>
     <fill>
@@ -144,12 +144,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDE3D2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002C4A3B"/>
+        <fgColor rgb="00141414"/>
       </patternFill>
     </fill>
   </fills>
@@ -179,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,13 +220,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -239,6 +231,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -250,24 +245,20 @@
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -703,7 +694,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Share taken by the 9 new colours</t>
+          <t>Share taken by the 8 new colours</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -1109,7 +1100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1124,7 +1115,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>THE 9 NEW AUTUMN / WINTER COLOURWAYS</t>
+          <t>THE 8 NEW AUTUMN / WINTER COLOURWAYS</t>
         </is>
       </c>
     </row>
@@ -1178,20 +1169,24 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Heather Grey Marl</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
+          <t>Marled yarn</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>#1F2A44</t>
-        </is>
-      </c>
-      <c r="E5" s="22" t="inlineStr"/>
+          <t>#9A9A9A</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>#4A4A4A</t>
+        </is>
+      </c>
       <c r="F5" s="12" t="n">
         <v>0.18</v>
       </c>
@@ -1206,7 +1201,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Grey Camo</t>
+          <t>Black Leopard</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -1216,16 +1211,16 @@
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>#8E9094</t>
+          <t>#111111</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>#3C3E42</t>
+          <t>#2E2A26</t>
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="G6" s="15">
         <f>ROUND(Assumptions!$B$7*Assumptions!$B$6*F6/10,0)*10</f>
@@ -1238,22 +1233,22 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Heather Grey Marl</t>
+          <t>Grey Leopard / Snow Leopard</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Marled yarn</t>
+          <t>Knitted jacquard</t>
         </is>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>#9A9A9A</t>
+          <t>#B9B7B2</t>
         </is>
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>#4A4A4A</t>
+          <t>#3A3A3A</t>
         </is>
       </c>
       <c r="F7" s="12" t="n">
@@ -1270,22 +1265,26 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Espresso Brown</t>
+          <t>Grey Camo</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
+          <t>Knitted jacquard</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>#4A342A</t>
-        </is>
-      </c>
-      <c r="E8" s="22" t="inlineStr"/>
+          <t>#8E9094</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>#3C3E42</t>
+        </is>
+      </c>
       <c r="F8" s="12" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="G8" s="15">
         <f>ROUND(Assumptions!$B$7*Assumptions!$B$6*F8/10,0)*10</f>
@@ -1298,7 +1297,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Terracotta</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
@@ -1308,12 +1307,12 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>#B0603C</t>
+          <t>#1F2A44</t>
         </is>
       </c>
       <c r="E9" s="22" t="inlineStr"/>
       <c r="F9" s="12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="G9" s="15">
         <f>ROUND(Assumptions!$B$7*Assumptions!$B$6*F9/10,0)*10</f>
@@ -1326,22 +1325,26 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Burgundy Wine</t>
+          <t>Cow Print</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
+          <t>Knitted jacquard</t>
         </is>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>#6E2233</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="inlineStr"/>
+          <t>#F2EFE9</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>#141414</t>
+        </is>
+      </c>
       <c r="F10" s="12" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="G10" s="15">
         <f>ROUND(Assumptions!$B$7*Assumptions!$B$6*F10/10,0)*10</f>
@@ -1386,7 +1389,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Nordic Fair Isle</t>
+          <t>Houndstooth Black / White</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -1396,12 +1399,12 @@
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>#EDE3D2</t>
+          <t>#141414</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>#A32234 / #22304A / #33352F</t>
+          <t>#F2EFE9</t>
         </is>
       </c>
       <c r="F12" s="12" t="n">
@@ -1413,52 +1416,24 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Forest Green</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="D13" s="30" t="inlineStr">
-        <is>
-          <t>#2C4A3B</t>
-        </is>
-      </c>
-      <c r="E13" s="22" t="inlineStr"/>
-      <c r="F13" s="12" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="G13" s="15">
-        <f>ROUND(Assumptions!$B$7*Assumptions!$B$6*F13/10,0)*10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G14" s="18">
-        <f>SUM(G5:G13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="31" t="inlineStr">
+      <c r="G13" s="18">
+        <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>GRAND TOTAL (restock + new)</t>
         </is>
       </c>
-      <c r="G16" s="7">
-        <f>'1 - Restock URGENT'!$E$13+'2 - New colourways'!$G$14</f>
+      <c r="G15" s="7">
+        <f>'1 - Restock URGENT'!$E$13+'2 - New colourways'!$G$13</f>
         <v/>
       </c>
     </row>
@@ -1473,7 +1448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1573,23 +1548,23 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>RESTOCK</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n"/>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="33" t="n"/>
-      <c r="F5" s="33" t="n"/>
-      <c r="G5" s="33" t="n"/>
-      <c r="H5" s="33" t="n"/>
-      <c r="I5" s="33" t="n"/>
-      <c r="J5" s="33" t="n"/>
-      <c r="K5" s="33" t="n"/>
-      <c r="L5" s="33" t="n"/>
-      <c r="M5" s="33" t="n"/>
+      <c r="B5" s="32" t="n"/>
+      <c r="C5" s="32" t="n"/>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="32" t="n"/>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="32" t="n"/>
+      <c r="H5" s="32" t="n"/>
+      <c r="I5" s="32" t="n"/>
+      <c r="J5" s="32" t="n"/>
+      <c r="K5" s="32" t="n"/>
+      <c r="L5" s="32" t="n"/>
+      <c r="M5" s="32" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -2032,28 +2007,28 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>NEW COLOURWAYS</t>
         </is>
       </c>
-      <c r="B14" s="33" t="n"/>
-      <c r="C14" s="33" t="n"/>
-      <c r="D14" s="33" t="n"/>
-      <c r="E14" s="33" t="n"/>
-      <c r="F14" s="33" t="n"/>
-      <c r="G14" s="33" t="n"/>
-      <c r="H14" s="33" t="n"/>
-      <c r="I14" s="33" t="n"/>
-      <c r="J14" s="33" t="n"/>
-      <c r="K14" s="33" t="n"/>
-      <c r="L14" s="33" t="n"/>
-      <c r="M14" s="33" t="n"/>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="32" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="32" t="n"/>
+      <c r="F14" s="32" t="n"/>
+      <c r="G14" s="32" t="n"/>
+      <c r="H14" s="32" t="n"/>
+      <c r="I14" s="32" t="n"/>
+      <c r="J14" s="32" t="n"/>
+      <c r="K14" s="32" t="n"/>
+      <c r="L14" s="32" t="n"/>
+      <c r="M14" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Heather Grey Marl</t>
         </is>
       </c>
       <c r="B15" s="14">
@@ -2108,7 +2083,7 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Grey Camo</t>
+          <t>Black Leopard</t>
         </is>
       </c>
       <c r="B16" s="14">
@@ -2163,7 +2138,7 @@
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Heather Grey Marl</t>
+          <t>Grey Leopard / Snow Leopard</t>
         </is>
       </c>
       <c r="B17" s="14">
@@ -2218,7 +2193,7 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Espresso Brown</t>
+          <t>Grey Camo</t>
         </is>
       </c>
       <c r="B18" s="14">
@@ -2273,7 +2248,7 @@
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Terracotta</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="B19" s="14">
@@ -2328,7 +2303,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>Burgundy Wine</t>
+          <t>Cow Print</t>
         </is>
       </c>
       <c r="B20" s="14">
@@ -2438,7 +2413,7 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>Nordic Fair Isle</t>
+          <t>Houndstooth Black / White</t>
         </is>
       </c>
       <c r="B22" s="14">
@@ -2487,61 +2462,6 @@
       </c>
       <c r="M22" s="18">
         <f>SUM(B22:L22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>Forest Green</t>
-        </is>
-      </c>
-      <c r="B23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="C23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$C$11,0)</f>
-        <v/>
-      </c>
-      <c r="D23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$D$11,0)</f>
-        <v/>
-      </c>
-      <c r="E23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$E$11,0)</f>
-        <v/>
-      </c>
-      <c r="F23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$F$11,0)</f>
-        <v/>
-      </c>
-      <c r="G23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$G$11,0)</f>
-        <v/>
-      </c>
-      <c r="H23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$H$11,0)</f>
-        <v/>
-      </c>
-      <c r="I23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$I$11,0)</f>
-        <v/>
-      </c>
-      <c r="J23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$J$11,0)</f>
-        <v/>
-      </c>
-      <c r="K23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$K$11,0)</f>
-        <v/>
-      </c>
-      <c r="L23" s="14">
-        <f>ROUND('2 - New colourways'!$G$13*Assumptions!$L$11,0)</f>
-        <v/>
-      </c>
-      <c r="M23" s="18">
-        <f>SUM(B23:L23)</f>
         <v/>
       </c>
     </row>
@@ -2618,28 +2538,28 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Navy</t>
-        </is>
-      </c>
-      <c r="C4" s="34" t="inlineStr"/>
+          <t>Heather Grey Marl</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr"/>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>#1F2A44</t>
+          <t>#9A9A9A / #4A4A4A</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>Deep rich navy. Match the navy already in production on our Cloud Walk Classic (same dye lot if possible). Tone-on-tone, matte.</t>
-        </is>
-      </c>
-      <c r="G4" s="35" t="inlineStr">
-        <is>
-          <t>#2 colour on Cloud Walk Classic (1,753 prs) and on Free Stride. Missing on this style.</t>
+          <t>Marled yarn</t>
+        </is>
+      </c>
+      <c r="F4" s="34" t="inlineStr">
+        <is>
+          <t>Salt-and-pepper marled melange: light grey + mid grey + charcoal fibres spun together. A YARN effect, NOT a print, NOT stripes, NOT camouflage. The classic marled-sweater look.</t>
+        </is>
+      </c>
+      <c r="G4" s="34" t="inlineStr">
+        <is>
+          <t>The same yarn effect ('Multicolor') is 21.7% of the Cloud Walk's entire volume - 11,871 pairs, the single biggest colourway of the whole store. And it is the cheapest of the nine to make: a yarn, not a jacquard.</t>
         </is>
       </c>
     </row>
@@ -2649,13 +2569,13 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Grey Camo</t>
-        </is>
-      </c>
-      <c r="C5" s="36" t="inlineStr"/>
+          <t>Black Leopard</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr"/>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>#8E9094 / #3C3E42</t>
+          <t>#111111 / #2E2A26</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -2663,14 +2583,14 @@
           <t>Knitted jacquard</t>
         </is>
       </c>
-      <c r="F5" s="35" t="inlineStr">
-        <is>
-          <t>Soft camouflage in FOUR GREYS ONLY: off-white, light grey, mid grey, charcoal. Rounded organic blotches approx 3-4 cm, soft edges, knitted in. STRICTLY greyscale - no green, no olive, no khaki, no brown.</t>
-        </is>
-      </c>
-      <c r="G5" s="35" t="inlineStr">
-        <is>
-          <t>Patterned neutrals are 30% of this style's volume (Leopard Brown 15% + Leopard Beige 10% + Checkered 5%). Grey camo is the same behaviour with a new look.</t>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>SAME leopard pattern and SAME spot scale as our existing Leopard Brown, recoloured tonal black: deep black base with jet-black and dark charcoal rosettes. Reads black at a distance, reveals the leopard up close. No brown, no tan, no gold.</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>Our #1 colour (Black, 32%) crossed with our #1 pattern family (leopard, 25% across two colourways). Same jacquard we already run, so no new development.</t>
         </is>
       </c>
     </row>
@@ -2680,28 +2600,28 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Heather Grey Marl</t>
-        </is>
-      </c>
-      <c r="C6" s="37" t="inlineStr"/>
+          <t>Grey Leopard / Snow Leopard</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="inlineStr"/>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>#9A9A9A / #4A4A4A</t>
+          <t>#B9B7B2 / #3A3A3A</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Marled yarn</t>
-        </is>
-      </c>
-      <c r="F6" s="35" t="inlineStr">
-        <is>
-          <t>Salt-and-pepper marled melange: light grey + mid grey + charcoal fibres spun together. A YARN effect, NOT a print, NOT stripes.</t>
-        </is>
-      </c>
-      <c r="G6" s="35" t="inlineStr">
-        <is>
-          <t>'Multicolor' (grey marl) is the best-selling colourway of the whole store on Cloud Walk. This style only has flat Grey today.</t>
+          <t>Knitted jacquard</t>
+        </is>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>SAME leopard pattern and SAME spot scale as our existing Leopard Brown, recoloured: light dove grey base with mid grey and charcoal rosettes. STRICTLY greyscale - no brown, no beige, no tan, no gold.</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>Leopard already runs in Brown (15%) and Beige (10%). Grey is our #2 colour and the obvious missing third. Same jacquard, new palette.</t>
         </is>
       </c>
     </row>
@@ -2711,28 +2631,28 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Espresso Brown</t>
-        </is>
-      </c>
-      <c r="C7" s="38" t="inlineStr"/>
+          <t>Grey Camo</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr"/>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>#4A342A</t>
+          <t>#8E9094 / #3C3E42</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
-        <is>
-          <t>Deep dark chocolate / espresso. Not tan, not caramel, not taupe.</t>
-        </is>
-      </c>
-      <c r="G7" s="35" t="inlineStr">
-        <is>
-          <t>442 prs on Cloud Walk Classic. Brown is the #1 AW26 footwear colour; pairs with Leopard Brown, our #3 here.</t>
+          <t>Knitted jacquard</t>
+        </is>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>Camouflage in FOUR GREYS ONLY: off-white, light grey, mid grey, charcoal. Rounded organic blotches approx 3-4 cm, soft edges, knitted in. STRICTLY greyscale - no green, no olive, no khaki, no brown.</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
+        <is>
+          <t>Patterned neutrals are 31% of this style's volume. Camo is the same buying behaviour as leopard with a new look, and a simple 4-colour jacquard.</t>
         </is>
       </c>
     </row>
@@ -2742,13 +2662,13 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Terracotta</t>
-        </is>
-      </c>
-      <c r="C8" s="39" t="inlineStr"/>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr"/>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>#B0603C</t>
+          <t>#1F2A44</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -2756,14 +2676,14 @@
           <t>Solid</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
-        <is>
-          <t>Warm burnt terracotta / rust. Earthy orange-brown, not neon, not coral.</t>
-        </is>
-      </c>
-      <c r="G8" s="35" t="inlineStr">
-        <is>
-          <t>491 prs on Cloud Walk Classic - ahead of Grey on that style. Signature autumn shade.</t>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>Deep rich navy. Match the navy already in production on our Cloud Walk Classic (same dye lot if possible). Tone-on-tone, matte.</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="inlineStr">
+        <is>
+          <t>The only solid worth adding: #2 colour on Cloud Walk Classic (22%), 2,968 prs on Cloud Walk, strong on Free Stride. Missing on this style.</t>
         </is>
       </c>
     </row>
@@ -2773,28 +2693,28 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Burgundy Wine</t>
-        </is>
-      </c>
-      <c r="C9" s="40" t="inlineStr"/>
+          <t>Cow Print</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr"/>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>#6E2233</t>
+          <t>#F2EFE9 / #141414</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="F9" s="35" t="inlineStr">
-        <is>
-          <t>Deep burgundy wine red. Blue-red, not orange-red, not bright red.</t>
-        </is>
-      </c>
-      <c r="G9" s="35" t="inlineStr">
-        <is>
-          <t>Plum Purple did 350 prs on Cloud Walk Classic: the deep red-purple family works on our buyer. Burgundy is the AW slipper classic.</t>
+          <t>Knitted jacquard</t>
+        </is>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>Holstein cow print: large irregular soft-edged BLACK blotches on a clean OFF-WHITE base. Big bold shapes approx 4-6 cm with plenty of space between them - NOT small dots, NOT leopard spots, NOT a busy speckle. Two colours only, knitted in.</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>The other big animal neutral in US loungewear for this buyer, and the simplest jacquard of the lot: two colours, big shapes. Loudest of the nine in an ad thumbnail.</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2727,7 @@
           <t>Buffalo Check Red / Black</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr"/>
+      <c r="C10" s="40" t="inlineStr"/>
       <c r="D10" s="22" t="inlineStr">
         <is>
           <t>#C1272D / #1A1A1A</t>
@@ -2818,14 +2738,14 @@
           <t>Knitted jacquard</t>
         </is>
       </c>
-      <c r="F10" s="35" t="inlineStr">
-        <is>
-          <t>Classic buffalo check: even squares approx 2 cm, true red x black, knitted in (jacquard), grid following the curve of the last. Collar SOLID BLACK.</t>
-        </is>
-      </c>
-      <c r="G10" s="35" t="inlineStr">
-        <is>
-          <t>The #1 classic of the US cosy-slipper category and the biggest Christmas gifting driver. We already run a check on this style.</t>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>Classic buffalo check: even squares approx 2 cm, true red x black, knitted in, grid following the curve of the last. Collar SOLID BLACK.</t>
+        </is>
+      </c>
+      <c r="G10" s="34" t="inlineStr">
+        <is>
+          <t>The #1 classic of the US cosy-slipper category and the main Christmas gifting driver. Same construction family as our existing Checkered.</t>
         </is>
       </c>
     </row>
@@ -2835,13 +2755,13 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Nordic Fair Isle</t>
-        </is>
-      </c>
-      <c r="C11" s="42" t="inlineStr"/>
+          <t>Houndstooth Black / White</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr"/>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>#EDE3D2 / #A32234 / #22304A / #33352F</t>
+          <t>#141414 / #F2EFE9</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -2849,120 +2769,97 @@
           <t>Knitted jacquard</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
-        <is>
-          <t>Cream / oatmeal base. Horizontal jacquard bands of snowflake + diamond motifs across the instep in deep red, navy, charcoal, with peerie dot rows between. Toe and heel SOLID CREAM. Knitted in, NOT printed, NOT embroidered.</t>
-        </is>
-      </c>
-      <c r="G11" s="35" t="inlineStr">
-        <is>
-          <t>The #1 winter knit pattern and the strongest gifting story for Nov-Dec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="66" customHeight="1">
-      <c r="A12" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Forest Green</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="inlineStr"/>
-      <c r="D12" s="22" t="inlineStr">
-        <is>
-          <t>#2C4A3B</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="F12" s="35" t="inlineStr">
-        <is>
-          <t>Deep dark blue-green pine forest green. CRITICAL: must NOT read olive, khaki, sage or army green - those are our two worst-selling colours ever.</t>
-        </is>
-      </c>
-      <c r="G12" s="35" t="inlineStr">
-        <is>
-          <t>236 prs on Cloud Walk Classic. Jewel green is a top AW26 runway colour. Smallest bet of the nine.</t>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>Classic pied-de-poule broken check, black and off-white, knitted in, BOLD scale of approx 2.5-3 cm per motif so it stays legible - not a fine micro houndstooth. Two colours. Collar SOLID BLACK.</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
+        <is>
+          <t>The geometric classic. Our Checkered proves two-tone geometric knits work here (3% on the shoe, 5% on the slipper); houndstooth is the same construction with a dressier repeat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t>PRODUCTION NOTES</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="44" t="inlineStr">
-        <is>
-          <t>PRODUCTION NOTES</t>
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>1. Last, construction, sole unit, insole, sizing and packaging: unchanged from current production. Colour is the only variable.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="45" t="inlineStr">
-        <is>
-          <t>1. Last, construction, sole unit, insole, sizing and packaging: unchanged from current production. Colour is the only variable.</t>
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>2. Lab dips required on all solid colourways before bulk - 3 options each (target / lighter / darker).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="45" t="inlineStr">
-        <is>
-          <t>2. Lab dips required on all solid colourways before bulk - 3 options each (target / lighter / darker).</t>
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>3. Knitted strike-offs required on the 7 patterned colourways (Heather Grey Marl, Black Leopard, Grey Leopard, Grey Camo, Cow Print, Buffalo Check, Houndstooth) before bulk. Patterns must be KNITTED IN, not printed and not embroidered.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="45" t="inlineStr">
-        <is>
-          <t>3. Knitted strike-offs required on the 4 patterned colourways (Grey Camo, Heather Grey Marl, Buffalo Check, Nordic Fair Isle) before bulk. Patterns must be KNITTED IN, not printed and not embroidered.</t>
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>4. HEX values are the visual target for the yarn dye. Pantone TCX to be confirmed on the approved lab dip.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="45" t="inlineStr">
-        <is>
-          <t>4. HEX values are the visual target for the yarn dye. Pantone TCX to be confirmed on the approved lab dip.</t>
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>5. Navy: please match the navy already running on our Cloud Walk Classic rather than creating a new shade.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="45" t="inlineStr">
-        <is>
-          <t>5. Navy: please match the navy already running on our Cloud Walk Classic rather than creating a new shade.</t>
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>6. Grey Camo and Grey Leopard must be STRICTLY greyscale. Any drift to olive, khaki, sage, army green, brown or tan will be rejected - those shades do not sell for us.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="45" t="inlineStr">
-        <is>
-          <t>6. Grey Camo must be STRICTLY greyscale and Forest Green must be a DEEP BLUE-GREEN. Any drift to olive / khaki / sage / army green will be rejected - those shades do not sell for us.</t>
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>6b. Black Leopard and Grey Leopard must reuse the EXACT leopard artwork and spot scale of our existing Leopard Brown - recolour only, no new engraving.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="A21" s="43" t="inlineStr">
         <is>
           <t>7. Colour fastness to rubbing and washing on the dark shades: no crocking onto light flooring or onto socks.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="inlineStr">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>8. Delivery target: 1 October 2026. Please confirm what is achievable by that date and what would land later - we will split the order accordingly.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="45" t="inlineStr">
+      <c r="A23" s="43" t="inlineStr">
         <is>
           <t>9. Please confirm: unit price per colourway, MOQ per colour and per size, lab dip / strike-off lead time, bulk lead time ex-works.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A18:G18"/>

</xml_diff>